<commit_message>
Schedule grid: 15-minute slots starting at noon
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JKLDuqsSkgnnSvq6gssh82
</commit_message>
<xml_diff>
--- a/docs/weekly-lesson-schedule.xlsx
+++ b/docs/weekly-lesson-schedule.xlsx
@@ -699,7 +699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -825,16 +825,20 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1">
+    <row r="6" ht="18" customHeight="1">
       <c r="A6" s="12" t="n">
-        <v>0.2916666666666667</v>
+        <v>0.5</v>
       </c>
       <c r="B6" s="13" t="n"/>
       <c r="C6" s="13" t="n"/>
       <c r="D6" s="13" t="n"/>
       <c r="E6" s="13" t="n"/>
       <c r="F6" s="13" t="n"/>
-      <c r="G6" s="13" t="n"/>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>BLOCKED – Travel tourney</t>
+        </is>
+      </c>
       <c r="H6" s="13" t="n"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
@@ -842,9 +846,9 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
+    <row r="7" ht="18" customHeight="1">
       <c r="A7" s="15" t="n">
-        <v>0.3125</v>
+        <v>0.5104166666666666</v>
       </c>
       <c r="B7" s="13" t="n"/>
       <c r="C7" s="13" t="n"/>
@@ -859,20 +863,16 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="12" t="n">
-        <v>0.3333333333333333</v>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="15" t="n">
+        <v>0.5208333333333334</v>
       </c>
       <c r="B8" s="13" t="n"/>
       <c r="C8" s="13" t="n"/>
       <c r="D8" s="13" t="n"/>
       <c r="E8" s="13" t="n"/>
       <c r="F8" s="13" t="n"/>
-      <c r="G8" s="13" t="inlineStr">
-        <is>
-          <t>BLOCKED – Travel tourney</t>
-        </is>
-      </c>
+      <c r="G8" s="13" t="n"/>
       <c r="H8" s="13" t="n"/>
       <c r="J8" s="17" t="inlineStr">
         <is>
@@ -880,9 +880,9 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
+    <row r="9" ht="18" customHeight="1">
       <c r="A9" s="15" t="n">
-        <v>0.3541666666666667</v>
+        <v>0.53125</v>
       </c>
       <c r="B9" s="13" t="n"/>
       <c r="C9" s="13" t="n"/>
@@ -897,9 +897,9 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
+    <row r="10" ht="18" customHeight="1">
       <c r="A10" s="12" t="n">
-        <v>0.375</v>
+        <v>0.5416666666666666</v>
       </c>
       <c r="B10" s="13" t="n"/>
       <c r="C10" s="13" t="n"/>
@@ -914,9 +914,9 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
+    <row r="11" ht="18" customHeight="1">
       <c r="A11" s="15" t="n">
-        <v>0.3958333333333333</v>
+        <v>0.5520833333333334</v>
       </c>
       <c r="B11" s="13" t="n"/>
       <c r="C11" s="13" t="n"/>
@@ -931,15 +931,11 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="12" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Jake M – Hitting</t>
-        </is>
-      </c>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="15" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="B12" s="13" t="n"/>
       <c r="C12" s="13" t="n"/>
       <c r="D12" s="13" t="n"/>
       <c r="E12" s="13" t="n"/>
@@ -947,15 +943,11 @@
       <c r="G12" s="13" t="n"/>
       <c r="H12" s="13" t="n"/>
     </row>
-    <row r="13" ht="22" customHeight="1">
+    <row r="13" ht="18" customHeight="1">
       <c r="A13" s="15" t="n">
-        <v>0.4375</v>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>Jake M – Hitting</t>
-        </is>
-      </c>
+        <v>0.5729166666666666</v>
+      </c>
+      <c r="B13" s="13" t="n"/>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="13" t="n"/>
       <c r="E13" s="13" t="n"/>
@@ -964,13 +956,13 @@
       <c r="H13" s="13" t="n"/>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>Tip: a lesson longer than 30 min —</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
+          <t>Tip: a lesson longer than 15 min —</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
       <c r="A14" s="12" t="n">
-        <v>0.4583333333333333</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="B14" s="13" t="n"/>
       <c r="C14" s="13" t="n"/>
@@ -985,9 +977,9 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
+    <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="n">
-        <v>0.4791666666666667</v>
+        <v>0.59375</v>
       </c>
       <c r="B15" s="13" t="n"/>
       <c r="C15" s="13" t="n"/>
@@ -997,9 +989,9 @@
       <c r="G15" s="13" t="n"/>
       <c r="H15" s="13" t="n"/>
     </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="12" t="n">
-        <v>0.5</v>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="15" t="n">
+        <v>0.6041666666666666</v>
       </c>
       <c r="B16" s="13" t="n"/>
       <c r="C16" s="13" t="n"/>
@@ -1009,9 +1001,9 @@
       <c r="G16" s="13" t="n"/>
       <c r="H16" s="13" t="n"/>
     </row>
-    <row r="17" ht="22" customHeight="1">
+    <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="n">
-        <v>0.5208333333333334</v>
+        <v>0.6145833333333334</v>
       </c>
       <c r="B17" s="13" t="n"/>
       <c r="C17" s="13" t="n"/>
@@ -1021,9 +1013,9 @@
       <c r="G17" s="13" t="n"/>
       <c r="H17" s="13" t="n"/>
     </row>
-    <row r="18" ht="22" customHeight="1">
+    <row r="18" ht="18" customHeight="1">
       <c r="A18" s="12" t="n">
-        <v>0.5416666666666666</v>
+        <v>0.625</v>
       </c>
       <c r="B18" s="13" t="n"/>
       <c r="C18" s="13" t="n"/>
@@ -1033,9 +1025,9 @@
       <c r="G18" s="13" t="n"/>
       <c r="H18" s="13" t="n"/>
     </row>
-    <row r="19" ht="22" customHeight="1">
+    <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="n">
-        <v>0.5625</v>
+        <v>0.6354166666666666</v>
       </c>
       <c r="B19" s="13" t="n"/>
       <c r="C19" s="13" t="n"/>
@@ -1045,9 +1037,9 @@
       <c r="G19" s="13" t="n"/>
       <c r="H19" s="13" t="n"/>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="12" t="n">
-        <v>0.5833333333333334</v>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="15" t="n">
+        <v>0.6458333333333334</v>
       </c>
       <c r="B20" s="13" t="n"/>
       <c r="C20" s="13" t="n"/>
@@ -1057,9 +1049,9 @@
       <c r="G20" s="13" t="n"/>
       <c r="H20" s="13" t="n"/>
     </row>
-    <row r="21" ht="22" customHeight="1">
+    <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="n">
-        <v>0.6041666666666666</v>
+        <v>0.65625</v>
       </c>
       <c r="B21" s="13" t="n"/>
       <c r="C21" s="13" t="n"/>
@@ -1069,11 +1061,15 @@
       <c r="G21" s="13" t="n"/>
       <c r="H21" s="13" t="n"/>
     </row>
-    <row r="22" ht="22" customHeight="1">
+    <row r="22" ht="18" customHeight="1">
       <c r="A22" s="12" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="B22" s="13" t="n"/>
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Jake M – Hitting</t>
+        </is>
+      </c>
       <c r="C22" s="13" t="n"/>
       <c r="D22" s="13" t="n"/>
       <c r="E22" s="13" t="n"/>
@@ -1081,11 +1077,15 @@
       <c r="G22" s="13" t="n"/>
       <c r="H22" s="13" t="n"/>
     </row>
-    <row r="23" ht="22" customHeight="1">
+    <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="n">
-        <v>0.6458333333333334</v>
-      </c>
-      <c r="B23" s="13" t="n"/>
+        <v>0.6770833333333334</v>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Jake M – Hitting</t>
+        </is>
+      </c>
       <c r="C23" s="13" t="n"/>
       <c r="D23" s="13" t="n"/>
       <c r="E23" s="13" t="n"/>
@@ -1093,11 +1093,15 @@
       <c r="G23" s="13" t="n"/>
       <c r="H23" s="13" t="n"/>
     </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="12" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="B24" s="13" t="n"/>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="15" t="n">
+        <v>0.6875</v>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Jake M – Hitting</t>
+        </is>
+      </c>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -1105,11 +1109,15 @@
       <c r="G24" s="13" t="n"/>
       <c r="H24" s="13" t="n"/>
     </row>
-    <row r="25" ht="22" customHeight="1">
+    <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="n">
-        <v>0.6875</v>
-      </c>
-      <c r="B25" s="13" t="n"/>
+        <v>0.6979166666666666</v>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>Jake M – Hitting</t>
+        </is>
+      </c>
       <c r="C25" s="13" t="n"/>
       <c r="D25" s="13" t="n"/>
       <c r="E25" s="13" t="n"/>
@@ -1117,7 +1125,7 @@
       <c r="G25" s="13" t="n"/>
       <c r="H25" s="13" t="n"/>
     </row>
-    <row r="26" ht="22" customHeight="1">
+    <row r="26" ht="18" customHeight="1">
       <c r="A26" s="12" t="n">
         <v>0.7083333333333334</v>
       </c>
@@ -1133,21 +1141,25 @@
       <c r="G26" s="13" t="n"/>
       <c r="H26" s="13" t="n"/>
     </row>
-    <row r="27" ht="22" customHeight="1">
+    <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="n">
-        <v>0.7291666666666666</v>
+        <v>0.71875</v>
       </c>
       <c r="B27" s="13" t="n"/>
       <c r="C27" s="13" t="n"/>
-      <c r="D27" s="13" t="n"/>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>Ava R – Pitching</t>
+        </is>
+      </c>
       <c r="E27" s="13" t="n"/>
       <c r="F27" s="13" t="n"/>
       <c r="G27" s="13" t="n"/>
       <c r="H27" s="13" t="n"/>
     </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="12" t="n">
-        <v>0.75</v>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="15" t="n">
+        <v>0.7291666666666666</v>
       </c>
       <c r="B28" s="13" t="n"/>
       <c r="C28" s="13" t="n"/>
@@ -1157,9 +1169,9 @@
       <c r="G28" s="13" t="n"/>
       <c r="H28" s="13" t="n"/>
     </row>
-    <row r="29" ht="22" customHeight="1">
+    <row r="29" ht="18" customHeight="1">
       <c r="A29" s="15" t="n">
-        <v>0.7708333333333334</v>
+        <v>0.7395833333333334</v>
       </c>
       <c r="B29" s="13" t="n"/>
       <c r="C29" s="13" t="n"/>
@@ -1169,9 +1181,9 @@
       <c r="G29" s="13" t="n"/>
       <c r="H29" s="13" t="n"/>
     </row>
-    <row r="30" ht="22" customHeight="1">
+    <row r="30" ht="18" customHeight="1">
       <c r="A30" s="12" t="n">
-        <v>0.7916666666666666</v>
+        <v>0.75</v>
       </c>
       <c r="B30" s="13" t="n"/>
       <c r="C30" s="13" t="n"/>
@@ -1181,9 +1193,9 @@
       <c r="G30" s="13" t="n"/>
       <c r="H30" s="13" t="n"/>
     </row>
-    <row r="31" ht="22" customHeight="1">
+    <row r="31" ht="18" customHeight="1">
       <c r="A31" s="15" t="n">
-        <v>0.8125</v>
+        <v>0.7604166666666666</v>
       </c>
       <c r="B31" s="13" t="n"/>
       <c r="C31" s="13" t="n"/>
@@ -1193,9 +1205,9 @@
       <c r="G31" s="13" t="n"/>
       <c r="H31" s="13" t="n"/>
     </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="12" t="n">
-        <v>0.8333333333333334</v>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="15" t="n">
+        <v>0.7708333333333334</v>
       </c>
       <c r="B32" s="13" t="n"/>
       <c r="C32" s="13" t="n"/>
@@ -1205,9 +1217,9 @@
       <c r="G32" s="13" t="n"/>
       <c r="H32" s="13" t="n"/>
     </row>
-    <row r="33" ht="22" customHeight="1">
+    <row r="33" ht="18" customHeight="1">
       <c r="A33" s="15" t="n">
-        <v>0.8541666666666666</v>
+        <v>0.78125</v>
       </c>
       <c r="B33" s="13" t="n"/>
       <c r="C33" s="13" t="n"/>
@@ -1217,49 +1229,145 @@
       <c r="G33" s="13" t="n"/>
       <c r="H33" s="13" t="n"/>
     </row>
-    <row r="34">
-      <c r="A34" s="7" t="inlineStr">
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="12" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="B34" s="13" t="n"/>
+      <c r="C34" s="13" t="n"/>
+      <c r="D34" s="13" t="n"/>
+      <c r="E34" s="13" t="n"/>
+      <c r="F34" s="13" t="n"/>
+      <c r="G34" s="13" t="n"/>
+      <c r="H34" s="13" t="n"/>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="15" t="n">
+        <v>0.8020833333333334</v>
+      </c>
+      <c r="B35" s="13" t="n"/>
+      <c r="C35" s="13" t="n"/>
+      <c r="D35" s="13" t="n"/>
+      <c r="E35" s="13" t="n"/>
+      <c r="F35" s="13" t="n"/>
+      <c r="G35" s="13" t="n"/>
+      <c r="H35" s="13" t="n"/>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="15" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="B36" s="13" t="n"/>
+      <c r="C36" s="13" t="n"/>
+      <c r="D36" s="13" t="n"/>
+      <c r="E36" s="13" t="n"/>
+      <c r="F36" s="13" t="n"/>
+      <c r="G36" s="13" t="n"/>
+      <c r="H36" s="13" t="n"/>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="15" t="n">
+        <v>0.8229166666666666</v>
+      </c>
+      <c r="B37" s="13" t="n"/>
+      <c r="C37" s="13" t="n"/>
+      <c r="D37" s="13" t="n"/>
+      <c r="E37" s="13" t="n"/>
+      <c r="F37" s="13" t="n"/>
+      <c r="G37" s="13" t="n"/>
+      <c r="H37" s="13" t="n"/>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="12" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="B38" s="13" t="n"/>
+      <c r="C38" s="13" t="n"/>
+      <c r="D38" s="13" t="n"/>
+      <c r="E38" s="13" t="n"/>
+      <c r="F38" s="13" t="n"/>
+      <c r="G38" s="13" t="n"/>
+      <c r="H38" s="13" t="n"/>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="15" t="n">
+        <v>0.84375</v>
+      </c>
+      <c r="B39" s="13" t="n"/>
+      <c r="C39" s="13" t="n"/>
+      <c r="D39" s="13" t="n"/>
+      <c r="E39" s="13" t="n"/>
+      <c r="F39" s="13" t="n"/>
+      <c r="G39" s="13" t="n"/>
+      <c r="H39" s="13" t="n"/>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="15" t="n">
+        <v>0.8541666666666666</v>
+      </c>
+      <c r="B40" s="13" t="n"/>
+      <c r="C40" s="13" t="n"/>
+      <c r="D40" s="13" t="n"/>
+      <c r="E40" s="13" t="n"/>
+      <c r="F40" s="13" t="n"/>
+      <c r="G40" s="13" t="n"/>
+      <c r="H40" s="13" t="n"/>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="15" t="n">
+        <v>0.8645833333333334</v>
+      </c>
+      <c r="B41" s="13" t="n"/>
+      <c r="C41" s="13" t="n"/>
+      <c r="D41" s="13" t="n"/>
+      <c r="E41" s="13" t="n"/>
+      <c r="F41" s="13" t="n"/>
+      <c r="G41" s="13" t="n"/>
+      <c r="H41" s="13" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
         <is>
           <t>Slots booked</t>
         </is>
       </c>
-      <c r="B34" s="7">
-        <f>COUNTA(B6:B33)-COUNTIF(B6:B33,"*BLOCKED*")</f>
-        <v/>
-      </c>
-      <c r="C34" s="7">
-        <f>COUNTA(C6:C33)-COUNTIF(C6:C33,"*BLOCKED*")</f>
-        <v/>
-      </c>
-      <c r="D34" s="7">
-        <f>COUNTA(D6:D33)-COUNTIF(D6:D33,"*BLOCKED*")</f>
-        <v/>
-      </c>
-      <c r="E34" s="7">
-        <f>COUNTA(E6:E33)-COUNTIF(E6:E33,"*BLOCKED*")</f>
-        <v/>
-      </c>
-      <c r="F34" s="7">
-        <f>COUNTA(F6:F33)-COUNTIF(F6:F33,"*BLOCKED*")</f>
-        <v/>
-      </c>
-      <c r="G34" s="7">
-        <f>COUNTA(G6:G33)-COUNTIF(G6:G33,"*BLOCKED*")</f>
-        <v/>
-      </c>
-      <c r="H34" s="7">
-        <f>COUNTA(H6:H33)-COUNTIF(H6:H33,"*BLOCKED*")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="G35" s="4" t="inlineStr">
+      <c r="B42" s="7">
+        <f>COUNTA(B6:B41)-COUNTIF(B6:B41,"*BLOCKED*")</f>
+        <v/>
+      </c>
+      <c r="C42" s="7">
+        <f>COUNTA(C6:C41)-COUNTIF(C6:C41,"*BLOCKED*")</f>
+        <v/>
+      </c>
+      <c r="D42" s="7">
+        <f>COUNTA(D6:D41)-COUNTIF(D6:D41,"*BLOCKED*")</f>
+        <v/>
+      </c>
+      <c r="E42" s="7">
+        <f>COUNTA(E6:E41)-COUNTIF(E6:E41,"*BLOCKED*")</f>
+        <v/>
+      </c>
+      <c r="F42" s="7">
+        <f>COUNTA(F6:F41)-COUNTIF(F6:F41,"*BLOCKED*")</f>
+        <v/>
+      </c>
+      <c r="G42" s="7">
+        <f>COUNTA(G6:G41)-COUNTIF(G6:G41,"*BLOCKED*")</f>
+        <v/>
+      </c>
+      <c r="H42" s="7">
+        <f>COUNTA(H6:H41)-COUNTIF(H6:H41,"*BLOCKED*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="G43" s="4" t="inlineStr">
         <is>
           <t>Slots this week:</t>
         </is>
       </c>
-      <c r="H35" s="21">
-        <f>SUM(B34:H34)</f>
+      <c r="H43" s="21">
+        <f>SUM(B42:H42)</f>
         <v/>
       </c>
     </row>
@@ -1267,7 +1375,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <conditionalFormatting sqref="B6:H33">
+  <conditionalFormatting sqref="B6:H41">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>ISNUMBER(SEARCH("Hitting",B6))</formula>
     </cfRule>
@@ -1394,10 +1502,10 @@
         <v/>
       </c>
       <c r="C2" s="24" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="D2" s="24" t="n">
-        <v>0.4583333333333333</v>
+        <v>0.7083333333333334</v>
       </c>
       <c r="E2" s="23">
         <f>IF(OR(C2="",D2=""),"",ROUND((D2-C2)*1440,0))</f>

</xml_diff>